<commit_message>
feat: persistent config and onboarding tweaks
</commit_message>
<xml_diff>
--- a/sample-question.xlsx
+++ b/sample-question.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/evgeniyraev/Developer/Labolatory/GalacticBlackFriday/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EAFDA5B-259F-CF4B-B689-546FD5B7A42E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E60D9A14-04DC-7642-B397-A1CD7D7D1319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7360" yWindow="5400" windowWidth="25020" windowHeight="15640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7360" yWindow="5400" windowWidth="25020" windowHeight="15640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quiz" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="53">
   <si>
     <t>Question</t>
   </si>
@@ -140,9 +140,6 @@
     <t>Count</t>
   </si>
   <si>
-    <t>близлка</t>
-  </si>
-  <si>
     <t>бисквитка</t>
   </si>
   <si>
@@ -156,6 +153,33 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>Коя планета е наречена "планетата джудже"? </t>
+  </si>
+  <si>
+    <t>Планетата на маймуните </t>
+  </si>
+  <si>
+    <t>Няма такова нещо</t>
+  </si>
+  <si>
+    <t>Плутон </t>
+  </si>
+  <si>
+    <t>Кое е превозното средство на астронавтите в Космоса? </t>
+  </si>
+  <si>
+    <t>Пони </t>
+  </si>
+  <si>
+    <t>Космическа ракета </t>
+  </si>
+  <si>
+    <t>Хеликоптер</t>
+  </si>
+  <si>
+    <t>близaлка</t>
   </si>
 </sst>
 </file>
@@ -539,161 +563,210 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="59.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>42</v>
-      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -722,18 +795,18 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B2">
         <v>0.6</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B3">
         <v>0.2</v>

</xml_diff>

<commit_message>
feat: add media tabs, working-hour playlist, and PIN screensaver
</commit_message>
<xml_diff>
--- a/sample-question.xlsx
+++ b/sample-question.xlsx
@@ -1,46 +1,227 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/evgeniyraev/Developer/Labolatory/GalacticBlackFriday/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34BEA83E-2EDC-F741-BF02-E81780AE665A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="880" windowWidth="41120" windowHeight="25700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Questions" sheetId="1" r:id="rId1"/>
     <sheet name="Awards" sheetId="2" r:id="rId2"/>
     <sheet name="NonWorking" sheetId="3" r:id="rId3"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
+  <si>
+    <t>Question</t>
+  </si>
+  <si>
+    <t>Answer A</t>
+  </si>
+  <si>
+    <t>Answer B</t>
+  </si>
+  <si>
+    <t>Answer C</t>
+  </si>
+  <si>
+    <t>Correct</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Award</t>
+  </si>
+  <si>
+    <t>Probability</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Video</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>afterhours/loop1.mp4</t>
+  </si>
+  <si>
+    <t>afterhours/loop2.mp4</t>
+  </si>
+  <si>
+    <t>afterhours/loop3.mp4</t>
+  </si>
+  <si>
+    <t>Кой е първият астронавт?​</t>
+  </si>
+  <si>
+    <t>АЛФ​</t>
+  </si>
+  <si>
+    <t>Юрий Гагарин​</t>
+  </si>
+  <si>
+    <t>Илън Мъск​</t>
+  </si>
+  <si>
+    <t>Кой известен спортист участва във филма „Космически забивки“?​</t>
+  </si>
+  <si>
+    <t>Майкъл Джордан​</t>
+  </si>
+  <si>
+    <t>Стефка Костадинова​</t>
+  </si>
+  <si>
+    <t>Соник​</t>
+  </si>
+  <si>
+    <t>Какво представлява млечният път?​</t>
+  </si>
+  <si>
+    <t>Спирална галактика в Слънчевата система. ​</t>
+  </si>
+  <si>
+    <t>Космически път, по който минава Голямата мечка.​</t>
+  </si>
+  <si>
+    <t>Пътеката на една гигантска крава в Космоса.​</t>
+  </si>
+  <si>
+    <t>Каква е основната причина Марс да изглежда червен?​</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Защото е срамежлив. ​</t>
+  </si>
+  <si>
+    <t>Защото е покрит с червен килим. ​</t>
+  </si>
+  <si>
+    <t>Има ръждясали железни частици в почвата.</t>
+  </si>
+  <si>
+    <t>Защо астронавтите тренират под вода?​</t>
+  </si>
+  <si>
+    <t> За да симулират безтегловност в контролирана среда.​</t>
+  </si>
+  <si>
+    <t>За да свикнат със срещи с русалки. ​</t>
+  </si>
+  <si>
+    <t>Защото НАСА тайно ги готви за „подводен космос“.​</t>
+  </si>
+  <si>
+    <t>Кое съзвездие съпътства Голямата мечка?​</t>
+  </si>
+  <si>
+    <t>Малката мечка​</t>
+  </si>
+  <si>
+    <t> Червената шапчица​</t>
+  </si>
+  <si>
+    <t>Костенурката нинджа​</t>
+  </si>
+  <si>
+    <t>Колко Луни има Земята?​</t>
+  </si>
+  <si>
+    <t>Една (нашата Луна). ​</t>
+  </si>
+  <si>
+    <t>Много – всяка нощ се сменят. ​</t>
+  </si>
+  <si>
+    <t>Пет, но четири са срамежливи и се крият. ​</t>
+  </si>
+  <si>
+    <t>На какво мирише Космоса според астронавтите? </t>
+  </si>
+  <si>
+    <t>На нищо - в Космоса няма въздух и миризма. </t>
+  </si>
+  <si>
+    <t>На горещ метал, барут или подобно. </t>
+  </si>
+  <si>
+    <t>На стари чорапи </t>
+  </si>
+  <si>
+    <t>Коя планета е наречена "планетата джудже"? </t>
+  </si>
+  <si>
+    <t>Планетата на маймуните </t>
+  </si>
+  <si>
+    <t>Няма такова нещо</t>
+  </si>
+  <si>
+    <t>Плутон </t>
+  </si>
+  <si>
+    <t>Кое е превозното средство на астронавтите в Космоса? </t>
+  </si>
+  <si>
+    <t>Пони </t>
+  </si>
+  <si>
+    <t>Космическа ракета </t>
+  </si>
+  <si>
+    <t>Хеликоптер</t>
+  </si>
+  <si>
+    <t>захарно петле</t>
+  </si>
+  <si>
+    <t>бисквитка</t>
+  </si>
+  <si>
+    <t>дъвка турбо</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -66,14 +247,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -398,114 +589,228 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Question</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Answer A</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Answer B</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Answer C</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Answer D</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Correct</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Which planet is known as the Red Planet?</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Mars</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Jupiter</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Saturn</v>
-      </c>
-      <c r="F2" t="str">
-        <v>B</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>How many moons does Earth have?</v>
-      </c>
-      <c r="B3" t="str">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E3" t="str">
-        <v>4</v>
-      </c>
-      <c r="F3" t="str">
-        <v>A</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Which gas is most abundant in the Earth's atmosphere?</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Oxygen</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Nitrogen</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Carbon Dioxide</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Hydrogen</v>
-      </c>
-      <c r="F4" t="str">
-        <v>B</v>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError sqref="A1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Award</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Probability</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Count</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Free Shore Excursion</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>56</v>
       </c>
       <c r="B2">
         <v>50</v>
@@ -514,9 +819,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Dinner with Captain</v>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>57</v>
       </c>
       <c r="B3">
         <v>30</v>
@@ -525,9 +830,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Spa Voucher</v>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>58</v>
       </c>
       <c r="B4">
         <v>20</v>
@@ -537,51 +842,58 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError sqref="A1:C1 B4:C4 B2:C2 B3:C3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Video</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Weight</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>afterhours/loop1.mp4</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>afterhours/loop2.mp4</v>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>13</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>afterhours/loop3.mp4</v>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>14</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+    <ignoredError sqref="A1:B4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>